<commit_message>
Admissions 360 package: label all deliverables 'Prepared for Management Review'
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PwvPj41jSev9ApGi3qLq4f
</commit_message>
<xml_diff>
--- a/pmu-admissions-audit/deliverables_360/02_PMU_Admissions_Content_Review_Register_EN.xlsx
+++ b/pmu-admissions-audit/deliverables_360/02_PMU_Admissions_Content_Review_Register_EN.xlsx
@@ -593,7 +593,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Prepared for management review. Not an approval, publication confirmation or closure certificate.</t>
+          <t>Prepared for Management Review. Not an approval, publication confirmation or closure certificate.</t>
         </is>
       </c>
     </row>
@@ -827,7 +827,7 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Ready for management review (draft, not approved)</t>
+          <t>Prepared for Management Review (not approved)</t>
         </is>
       </c>
     </row>

</xml_diff>